<commit_message>
làm các chức năng của tài chính
</commit_message>
<xml_diff>
--- a/public/templates/MauChamCong.xlsx
+++ b/public/templates/MauChamCong.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ThucTapOTruong\Code\hp-english-homestay\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7245A6CC-8104-4E4B-98E8-2DB647C0D26F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B69F64DE-3CC7-48F5-850A-88B1BAB5ABB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9FB942CE-C84A-480B-8E4F-5A0FA45B77FF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="36">
   <si>
     <t>Mã ID</t>
   </si>
@@ -1410,24 +1410,9 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39">
-        <v>39</v>
-      </c>
-      <c r="B39" t="s">
-        <v>16</v>
-      </c>
-      <c r="C39" t="s">
-        <v>35</v>
-      </c>
-      <c r="D39" s="1">
-        <v>46142</v>
-      </c>
-      <c r="E39" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F39" s="2">
-        <v>0.72916666666666663</v>
-      </c>
+      <c r="D39" s="1"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D40" s="1"/>

</xml_diff>

<commit_message>
thêm tính năng xem riêng phiếu lương của tài khoản
</commit_message>
<xml_diff>
--- a/public/templates/MauChamCong.xlsx
+++ b/public/templates/MauChamCong.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ThucTapOTruong\Code\hp-english-homestay\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B69F64DE-3CC7-48F5-850A-88B1BAB5ABB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F1A615-4F2B-4CA5-8495-12C280C0A6CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9FB942CE-C84A-480B-8E4F-5A0FA45B77FF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="38">
   <si>
     <t>Mã ID</t>
   </si>
@@ -144,13 +144,19 @@
   </si>
   <si>
     <t>Trần Thị Tuyết</t>
+  </si>
+  <si>
+    <t>GV3</t>
+  </si>
+  <si>
+    <t>David Smith</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -168,6 +174,13 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -199,7 +212,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -218,6 +231,7 @@
     <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -552,7 +566,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8A8993C-3A32-4025-A3CC-AB986AB30619}">
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.44140625" customWidth="1"/>
@@ -560,7 +574,7 @@
     <col min="4" max="4" width="11.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -610,7 +624,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -630,7 +644,7 @@
         <v>0.72916666666666663</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -650,61 +664,55 @@
         <v>0.72916666666666663</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D4" s="1">
-        <v>46115</v>
+        <v>46114</v>
       </c>
       <c r="E4" s="2">
-        <v>0.33124999999999999</v>
+        <v>0.38541666666666669</v>
       </c>
       <c r="F4" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+        <v>0.46875</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>33</v>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>35</v>
       </c>
       <c r="D5" s="1">
-        <v>46116</v>
+        <v>46115</v>
       </c>
       <c r="E5" s="2">
-        <v>0.33333333333333331</v>
+        <v>0.33124999999999999</v>
       </c>
       <c r="F5" s="2">
-        <v>0.50347222222222221</v>
-      </c>
-      <c r="G5" s="2">
-        <v>0.5625</v>
-      </c>
-      <c r="H5" s="2">
-        <v>0.8125</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>35</v>
+      <c r="B6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>33</v>
       </c>
       <c r="D6" s="1">
         <v>46116</v>
@@ -713,70 +721,78 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="F6" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+        <v>0.50347222222222221</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0.5625</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
-        <v>16</v>
+      <c r="B7" s="4" t="s">
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D7" s="1">
-        <v>46118</v>
+        <v>46116</v>
       </c>
       <c r="E7" s="2">
-        <v>0.33333333333333331</v>
+        <v>0.29166666666666669</v>
       </c>
       <c r="F7" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="D8" s="1">
-        <v>46119</v>
+        <v>46116</v>
       </c>
       <c r="E8" s="2">
-        <v>0.3888888888888889</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="F8" s="2">
-        <v>0.47222222222222221</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D9" s="1">
-        <v>46119</v>
+        <v>46146</v>
       </c>
       <c r="E9" s="2">
-        <v>0.33333333333333331</v>
+        <v>0.29166666666666669</v>
       </c>
       <c r="F9" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -787,7 +803,7 @@
         <v>35</v>
       </c>
       <c r="D10" s="1">
-        <v>46120</v>
+        <v>46118</v>
       </c>
       <c r="E10" s="2">
         <v>0.33333333333333331</v>
@@ -796,7 +812,7 @@
         <v>0.72916666666666663</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -804,19 +820,19 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D11" s="1">
-        <v>46121</v>
+        <v>46119</v>
       </c>
       <c r="E11" s="2">
-        <v>0.38194444444444442</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="F11" s="2">
         <v>0.47222222222222221</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -827,7 +843,7 @@
         <v>35</v>
       </c>
       <c r="D12" s="1">
-        <v>46121</v>
+        <v>46119</v>
       </c>
       <c r="E12" s="2">
         <v>0.33333333333333331</v>
@@ -836,7 +852,7 @@
         <v>0.72916666666666663</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -847,7 +863,7 @@
         <v>35</v>
       </c>
       <c r="D13" s="1">
-        <v>46122</v>
+        <v>46120</v>
       </c>
       <c r="E13" s="2">
         <v>0.33333333333333331</v>
@@ -856,7 +872,7 @@
         <v>0.72916666666666663</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -864,31 +880,19 @@
         <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D14" s="1">
-        <v>46123</v>
+        <v>46121</v>
       </c>
       <c r="E14" s="2">
-        <v>0.29166666666666669</v>
+        <v>0.38194444444444442</v>
       </c>
       <c r="F14" s="2">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="G14" s="2">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="H14" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-      <c r="I14" s="2">
-        <v>0.75</v>
-      </c>
-      <c r="J14" s="2">
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+        <v>0.47222222222222221</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -899,7 +903,7 @@
         <v>35</v>
       </c>
       <c r="D15" s="1">
-        <v>46123</v>
+        <v>46121</v>
       </c>
       <c r="E15" s="2">
         <v>0.33333333333333331</v>
@@ -907,215 +911,197 @@
       <c r="F15" s="2">
         <v>0.72916666666666663</v>
       </c>
-      <c r="R15" s="2"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="1">
+        <v>46122</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="1">
+        <v>46123</v>
+      </c>
+      <c r="E17" s="2">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="1">
+        <v>46123</v>
+      </c>
+      <c r="E18" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="R18" s="2"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
         <v>19</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C19" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D19" s="1">
         <v>46124</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E19" s="2">
         <v>0.29166666666666669</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F19" s="2">
         <v>0.375</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G19" s="2">
         <v>0.54166666666666663</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H19" s="2">
         <v>0.625</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" s="1">
+        <v>46124</v>
+      </c>
+      <c r="E20" s="2">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0.375</v>
+      </c>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
         <v>14</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C21" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D21" s="1">
         <v>46125</v>
       </c>
-      <c r="E17" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F17" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>18</v>
-      </c>
-      <c r="B18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" t="s">
-        <v>35</v>
-      </c>
-      <c r="D18" s="1">
+      <c r="E21" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F21" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22" s="1">
         <v>46125</v>
       </c>
-      <c r="E18" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F18" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>19</v>
-      </c>
-      <c r="B19" s="4" t="s">
+      <c r="E22" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F22" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" s="1">
+        <v>46116</v>
+      </c>
+      <c r="E23" s="2">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="F23" s="2">
+        <v>0.46875</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A24">
         <v>23</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="B24" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="D19" s="5">
-        <v>46126</v>
-      </c>
-      <c r="E19" s="6">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F19" s="6">
-        <v>0.72916666666666663</v>
-      </c>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>20</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D20" s="5">
-        <v>46126</v>
-      </c>
-      <c r="E20" s="6">
-        <v>0.375</v>
-      </c>
-      <c r="F20" s="6">
-        <v>0.73958333333333337</v>
-      </c>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>21</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D21" s="5">
-        <v>46126</v>
-      </c>
-      <c r="E21" s="6">
-        <v>0.3125</v>
-      </c>
-      <c r="F21" s="6">
-        <v>0.39583333333333331</v>
-      </c>
-      <c r="G21" s="6">
-        <v>0.5625</v>
-      </c>
-      <c r="H21" s="6">
-        <v>0.64583333333333337</v>
-      </c>
-      <c r="I21" s="6">
-        <v>0.72916666666666663</v>
-      </c>
-      <c r="J21" s="6">
-        <v>0.8125</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>22</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="5">
-        <v>46126</v>
-      </c>
-      <c r="E22" s="6">
-        <v>0.70833333333333337</v>
-      </c>
-      <c r="F22" s="6">
-        <v>0.875</v>
-      </c>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>23</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D23" s="5">
-        <v>46126</v>
-      </c>
-      <c r="E23" s="6">
-        <v>0.375</v>
-      </c>
-      <c r="F23" s="6">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="G23" s="6">
-        <v>0.75</v>
-      </c>
-      <c r="H23" s="6">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>24</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="D24" s="5">
         <v>46126</v>
@@ -1123,305 +1109,605 @@
       <c r="E24" s="6">
         <v>0.33333333333333331</v>
       </c>
-      <c r="F24" s="7"/>
+      <c r="F24" s="6">
+        <v>0.72916666666666663</v>
+      </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
       <c r="J24" s="4"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B25" t="s">
-        <v>16</v>
-      </c>
-      <c r="C25" t="s">
-        <v>35</v>
-      </c>
-      <c r="D25" s="1">
+      <c r="C25" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="5">
         <v>46126</v>
       </c>
-      <c r="E25" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F25" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="E25" s="6">
+        <v>0.375</v>
+      </c>
+      <c r="F25" s="6">
+        <v>0.73958333333333337</v>
+      </c>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B26" t="s">
-        <v>16</v>
-      </c>
-      <c r="C26" t="s">
-        <v>35</v>
-      </c>
-      <c r="D26" s="1">
+      <c r="C26" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D26" s="5">
+        <v>46126</v>
+      </c>
+      <c r="E26" s="6">
+        <v>0.3125</v>
+      </c>
+      <c r="F26" s="6">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="G26" s="6">
+        <v>0.5625</v>
+      </c>
+      <c r="H26" s="6">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="I26" s="6">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="J26" s="6">
+        <v>0.8125</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D27" s="5">
+        <v>46126</v>
+      </c>
+      <c r="E27" s="6">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F27" s="6">
+        <v>0.875</v>
+      </c>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D28" s="5">
+        <v>46126</v>
+      </c>
+      <c r="E28" s="6">
+        <v>0.375</v>
+      </c>
+      <c r="F28" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="G28" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="H28" s="6">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D29" s="5">
+        <v>46126</v>
+      </c>
+      <c r="E29" s="6">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F29" s="7"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" t="s">
+        <v>35</v>
+      </c>
+      <c r="D30" s="1">
+        <v>46126</v>
+      </c>
+      <c r="E30" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31" s="1">
         <v>46127</v>
       </c>
-      <c r="E26" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F26" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A27">
-        <v>27</v>
-      </c>
-      <c r="B27" t="s">
-        <v>16</v>
-      </c>
-      <c r="C27" t="s">
-        <v>35</v>
-      </c>
-      <c r="D27" s="1">
+      <c r="E31" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F31" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D32" s="1">
         <v>46128</v>
       </c>
-      <c r="E27" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F27" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A28">
-        <v>28</v>
-      </c>
-      <c r="B28" t="s">
-        <v>16</v>
-      </c>
-      <c r="C28" t="s">
-        <v>35</v>
-      </c>
-      <c r="D28" s="1">
+      <c r="E32" s="2">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="F32" s="2">
+        <v>0.46875</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" t="s">
+        <v>35</v>
+      </c>
+      <c r="D33" s="1">
+        <v>46128</v>
+      </c>
+      <c r="E33" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F33" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" t="s">
+        <v>35</v>
+      </c>
+      <c r="D34" s="1">
         <v>46129</v>
       </c>
-      <c r="E28" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F28" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A29">
-        <v>29</v>
-      </c>
-      <c r="B29" t="s">
-        <v>16</v>
-      </c>
-      <c r="C29" t="s">
-        <v>35</v>
-      </c>
-      <c r="D29" s="1">
+      <c r="E34" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F34" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" t="s">
+        <v>35</v>
+      </c>
+      <c r="D35" s="1">
         <v>46130</v>
       </c>
-      <c r="E29" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F29" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A30">
-        <v>30</v>
-      </c>
-      <c r="B30" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" t="s">
-        <v>35</v>
-      </c>
-      <c r="D30" s="1">
+      <c r="E35" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F35" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>17</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D36" s="1">
+        <v>46130</v>
+      </c>
+      <c r="E36" s="2">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="F36" s="2">
+        <v>0.46875</v>
+      </c>
+      <c r="G36" s="2">
+        <v>0.73958333333333337</v>
+      </c>
+      <c r="H36" s="2">
+        <v>0.82291666666666663</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>17</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D37" s="1">
+        <v>46131</v>
+      </c>
+      <c r="E37" s="2">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="F37" s="2">
+        <v>0.375</v>
+      </c>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>16</v>
+      </c>
+      <c r="C38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D38" s="1">
         <v>46132</v>
       </c>
-      <c r="E30" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F30" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A31">
-        <v>31</v>
-      </c>
-      <c r="B31" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31" t="s">
-        <v>35</v>
-      </c>
-      <c r="D31" s="1">
+      <c r="E38" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F38" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" t="s">
+        <v>35</v>
+      </c>
+      <c r="D39" s="1">
         <v>46133</v>
       </c>
-      <c r="E31" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F31" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A32">
-        <v>32</v>
-      </c>
-      <c r="B32" t="s">
-        <v>16</v>
-      </c>
-      <c r="C32" t="s">
-        <v>35</v>
-      </c>
-      <c r="D32" s="1">
+      <c r="E39" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F39" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>17</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D40" s="1">
+        <v>46133</v>
+      </c>
+      <c r="E40" s="2">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="F40" s="2">
+        <v>0.46875</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>16</v>
+      </c>
+      <c r="C41" t="s">
+        <v>35</v>
+      </c>
+      <c r="D41" s="1">
         <v>46134</v>
       </c>
-      <c r="E32" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F32" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33">
-        <v>33</v>
-      </c>
-      <c r="B33" t="s">
-        <v>16</v>
-      </c>
-      <c r="C33" t="s">
-        <v>35</v>
-      </c>
-      <c r="D33" s="1">
+      <c r="E41" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F41" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>16</v>
+      </c>
+      <c r="C42" t="s">
+        <v>35</v>
+      </c>
+      <c r="D42" s="1">
         <v>46135</v>
       </c>
-      <c r="E33" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F33" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34">
-        <v>34</v>
-      </c>
-      <c r="B34" t="s">
-        <v>16</v>
-      </c>
-      <c r="C34" t="s">
-        <v>35</v>
-      </c>
-      <c r="D34" s="1">
+      <c r="E42" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F42" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>17</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D43" s="1">
+        <v>46135</v>
+      </c>
+      <c r="E43" s="2">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="F43" s="2">
+        <v>0.46875</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" t="s">
+        <v>35</v>
+      </c>
+      <c r="D44" s="1">
         <v>46136</v>
       </c>
-      <c r="E34" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F34" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35">
-        <v>35</v>
-      </c>
-      <c r="B35" t="s">
-        <v>16</v>
-      </c>
-      <c r="C35" t="s">
-        <v>35</v>
-      </c>
-      <c r="D35" s="1">
+      <c r="E44" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F44" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>16</v>
+      </c>
+      <c r="C45" t="s">
+        <v>35</v>
+      </c>
+      <c r="D45" s="1">
         <v>46137</v>
       </c>
-      <c r="E35" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F35" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36">
-        <v>36</v>
-      </c>
-      <c r="B36" t="s">
-        <v>16</v>
-      </c>
-      <c r="C36" t="s">
-        <v>35</v>
-      </c>
-      <c r="D36" s="1">
+      <c r="E45" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F45" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D46" s="1">
+        <v>46137</v>
+      </c>
+      <c r="E46" s="2">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="F46" s="2">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D47" s="1">
+        <v>46138</v>
+      </c>
+      <c r="E47" s="2">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="F47" s="2">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>16</v>
+      </c>
+      <c r="C48" t="s">
+        <v>35</v>
+      </c>
+      <c r="D48" s="1">
         <v>46139</v>
       </c>
-      <c r="E36" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F36" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37">
+      <c r="E48" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F48" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" t="s">
+        <v>35</v>
+      </c>
+      <c r="D49" s="1">
+        <v>46140</v>
+      </c>
+      <c r="E49" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F49" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>17</v>
+      </c>
+      <c r="C50" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B37" t="s">
-        <v>16</v>
-      </c>
-      <c r="C37" t="s">
-        <v>35</v>
-      </c>
-      <c r="D37" s="1">
+      <c r="D50" s="1">
         <v>46140</v>
       </c>
-      <c r="E37" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F37" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38">
-        <v>38</v>
-      </c>
-      <c r="B38" t="s">
-        <v>16</v>
-      </c>
-      <c r="C38" t="s">
-        <v>35</v>
-      </c>
-      <c r="D38" s="1">
+      <c r="E50" s="2">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="F50" s="2">
+        <v>0.46875</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>16</v>
+      </c>
+      <c r="C51" t="s">
+        <v>35</v>
+      </c>
+      <c r="D51" s="1">
         <v>46141</v>
       </c>
-      <c r="E38" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F38" s="2">
-        <v>0.72916666666666663</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="D39" s="1"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="D40" s="1"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
+      <c r="E51" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F51" s="2">
+        <v>0.72916666666666663</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D52" s="1"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D53" s="1"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A39">
-    <sortCondition ref="A2:A39"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A52">
+    <sortCondition ref="A2:A52"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix tooltip chấm công
</commit_message>
<xml_diff>
--- a/public/templates/MauChamCong.xlsx
+++ b/public/templates/MauChamCong.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ThucTapOTruong\Code\hp-english-homestay\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F1A615-4F2B-4CA5-8495-12C280C0A6CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B6A449E-C711-460A-A37C-FA759D6E5EC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9FB942CE-C84A-480B-8E4F-5A0FA45B77FF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="37">
   <si>
     <t>Mã ID</t>
   </si>
@@ -144,9 +144,6 @@
   </si>
   <si>
     <t>Trần Thị Tuyết</t>
-  </si>
-  <si>
-    <t>GV3</t>
   </si>
   <si>
     <t>David Smith</t>
@@ -672,7 +669,7 @@
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="1">
         <v>46114</v>
@@ -735,10 +732,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
         <v>36</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
       </c>
       <c r="D7" s="1">
         <v>46116</v>
@@ -780,7 +777,7 @@
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" s="1">
         <v>46146</v>
@@ -820,13 +817,13 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D11" s="1">
         <v>46119</v>
       </c>
       <c r="E11" s="2">
-        <v>0.3888888888888889</v>
+        <v>0.38194444444444442</v>
       </c>
       <c r="F11" s="2">
         <v>0.47222222222222221</v>
@@ -880,7 +877,7 @@
         <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D14" s="1">
         <v>46121</v>
@@ -1019,7 +1016,7 @@
         <v>17</v>
       </c>
       <c r="C20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D20" s="1">
         <v>46124</v>
@@ -1081,7 +1078,7 @@
         <v>17</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D23" s="1">
         <v>46116</v>
@@ -1295,7 +1292,7 @@
         <v>17</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D32" s="1">
         <v>46128</v>
@@ -1375,7 +1372,7 @@
         <v>17</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D36" s="1">
         <v>46130</v>
@@ -1401,7 +1398,7 @@
         <v>17</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D37" s="1">
         <v>46131</v>
@@ -1463,7 +1460,7 @@
         <v>17</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D40" s="1">
         <v>46133</v>
@@ -1523,7 +1520,7 @@
         <v>17</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D43" s="1">
         <v>46135</v>
@@ -1583,7 +1580,7 @@
         <v>17</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D46" s="1">
         <v>46137</v>
@@ -1603,7 +1600,7 @@
         <v>17</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D47" s="1">
         <v>46138</v>
@@ -1663,7 +1660,7 @@
         <v>17</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D50" s="1">
         <v>46140</v>

</xml_diff>